<commit_message>
Add audience creation and upload workflow
</commit_message>
<xml_diff>
--- a/examples/meta_ads_workflow_template.xlsx
+++ b/examples/meta_ads_workflow_template.xlsx
@@ -12,11 +12,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AdSets" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creatives" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ads" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BulkChanges" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PerformanceSnapshots" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PublishLog" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ValidationErrors" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookups" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audiences" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudienceUploads" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BulkChanges" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PerformanceSnapshots" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PublishLog" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ValidationErrors" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookups" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -193,8 +195,47 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="LookupsTable" displayName="LookupsTable" ref="A1:B18" headerRowCount="1">
-  <autoFilter ref="A1:B18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="PublishLogTable" displayName="PublishLogTable" ref="A1:N2" headerRowCount="1">
+  <autoFilter ref="A1:N2"/>
+  <tableColumns count="14">
+    <tableColumn id="1" name="log_id"/>
+    <tableColumn id="2" name="timestamp"/>
+    <tableColumn id="3" name="mode"/>
+    <tableColumn id="4" name="action_id"/>
+    <tableColumn id="5" name="operation"/>
+    <tableColumn id="6" name="object_type"/>
+    <tableColumn id="7" name="object_key"/>
+    <tableColumn id="8" name="meta_id"/>
+    <tableColumn id="9" name="command"/>
+    <tableColumn id="10" name="payload_hash"/>
+    <tableColumn id="11" name="status"/>
+    <tableColumn id="12" name="message"/>
+    <tableColumn id="13" name="stdout"/>
+    <tableColumn id="14" name="stderr"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="ValidationErrorsTable" displayName="ValidationErrorsTable" ref="A1:G2" headerRowCount="1">
+  <autoFilter ref="A1:G2"/>
+  <tableColumns count="7">
+    <tableColumn id="1" name="validation_id"/>
+    <tableColumn id="2" name="timestamp"/>
+    <tableColumn id="3" name="severity"/>
+    <tableColumn id="4" name="table"/>
+    <tableColumn id="5" name="row_key"/>
+    <tableColumn id="6" name="field"/>
+    <tableColumn id="7" name="message"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="LookupsTable" displayName="LookupsTable" ref="A1:B25" headerRowCount="1">
+  <autoFilter ref="A1:B25"/>
   <tableColumns count="2">
     <tableColumn id="1" name="type"/>
     <tableColumn id="2" name="value"/>
@@ -320,7 +361,56 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="BulkChangesTable" displayName="BulkChangesTable" ref="A1:M4" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="AudiencesTable" displayName="AudiencesTable" ref="A1:T5" headerRowCount="1">
+  <autoFilter ref="A1:T5"/>
+  <tableColumns count="20">
+    <tableColumn id="1" name="audience_key"/>
+    <tableColumn id="2" name="account_key"/>
+    <tableColumn id="3" name="meta_audience_id"/>
+    <tableColumn id="4" name="name"/>
+    <tableColumn id="5" name="audience_type"/>
+    <tableColumn id="6" name="subtype"/>
+    <tableColumn id="7" name="description"/>
+    <tableColumn id="8" name="source_audience_key"/>
+    <tableColumn id="9" name="pixel_dataset_id"/>
+    <tableColumn id="10" name="retention_days"/>
+    <tableColumn id="11" name="countries"/>
+    <tableColumn id="12" name="lookalike_ratio"/>
+    <tableColumn id="13" name="targeting_json"/>
+    <tableColumn id="14" name="rule_json"/>
+    <tableColumn id="15" name="lookalike_spec_json"/>
+    <tableColumn id="16" name="customer_file_source"/>
+    <tableColumn id="17" name="approval_status"/>
+    <tableColumn id="18" name="last_result"/>
+    <tableColumn id="19" name="last_error"/>
+    <tableColumn id="20" name="updated_at"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="AudienceUploadsTable" displayName="AudienceUploadsTable" ref="A1:K2" headerRowCount="1">
+  <autoFilter ref="A1:K2"/>
+  <tableColumns count="11">
+    <tableColumn id="1" name="upload_key"/>
+    <tableColumn id="2" name="audience_key"/>
+    <tableColumn id="3" name="operation"/>
+    <tableColumn id="4" name="schema"/>
+    <tableColumn id="5" name="data_path"/>
+    <tableColumn id="6" name="data_json"/>
+    <tableColumn id="7" name="hash_type"/>
+    <tableColumn id="8" name="approval_status"/>
+    <tableColumn id="9" name="applied_at"/>
+    <tableColumn id="10" name="result"/>
+    <tableColumn id="11" name="error"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="BulkChangesTable" displayName="BulkChangesTable" ref="A1:M4" headerRowCount="1">
   <autoFilter ref="A1:M4"/>
   <tableColumns count="13">
     <tableColumn id="1" name="change_id"/>
@@ -341,8 +431,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="PerformanceSnapshotsTable" displayName="PerformanceSnapshotsTable" ref="A1:AB2" headerRowCount="1">
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="PerformanceSnapshotsTable" displayName="PerformanceSnapshotsTable" ref="A1:AB2" headerRowCount="1">
   <autoFilter ref="A1:AB2"/>
   <tableColumns count="28">
     <tableColumn id="1" name="snapshot_key"/>
@@ -373,45 +463,6 @@
     <tableColumn id="26" name="cpl"/>
     <tableColumn id="27" name="budget_utilization"/>
     <tableColumn id="28" name="pacing_ratio"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PublishLogTable" displayName="PublishLogTable" ref="A1:N2" headerRowCount="1">
-  <autoFilter ref="A1:N2"/>
-  <tableColumns count="14">
-    <tableColumn id="1" name="log_id"/>
-    <tableColumn id="2" name="timestamp"/>
-    <tableColumn id="3" name="mode"/>
-    <tableColumn id="4" name="action_id"/>
-    <tableColumn id="5" name="operation"/>
-    <tableColumn id="6" name="object_type"/>
-    <tableColumn id="7" name="object_key"/>
-    <tableColumn id="8" name="meta_id"/>
-    <tableColumn id="9" name="command"/>
-    <tableColumn id="10" name="payload_hash"/>
-    <tableColumn id="11" name="status"/>
-    <tableColumn id="12" name="message"/>
-    <tableColumn id="13" name="stdout"/>
-    <tableColumn id="14" name="stderr"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="ValidationErrorsTable" displayName="ValidationErrorsTable" ref="A1:G2" headerRowCount="1">
-  <autoFilter ref="A1:G2"/>
-  <tableColumns count="7">
-    <tableColumn id="1" name="validation_id"/>
-    <tableColumn id="2" name="timestamp"/>
-    <tableColumn id="3" name="severity"/>
-    <tableColumn id="4" name="table"/>
-    <tableColumn id="5" name="row_key"/>
-    <tableColumn id="6" name="field"/>
-    <tableColumn id="7" name="message"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -907,7 +958,177 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>log_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>timestamp</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>mode</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>action_id</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>operation</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>object_type</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>object_key</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>meta_id</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>command</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>payload_hash</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>stdout</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>stderr</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>validation_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>timestamp</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>severity</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>table</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>row_key</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1085,46 +1306,130 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>cta</t>
+          <t>audience_type</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>SHOP_NOW</t>
+          <t>CUSTOM</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>cta</t>
+          <t>audience_type</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>LEARN_MORE</t>
+          <t>LOOKALIKE</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>cta</t>
+          <t>audience_type</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>SIGN_UP</t>
+          <t>WEBSITE</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>audience_type</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>SAVED</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>audience_upload_operation</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>audience_upload_operation</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>REMOVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>audience_upload_operation</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>REPLACE</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
           <t>cta</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>SHOP_NOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>cta</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>LEARN_MORE</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>cta</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>SIGN_UP</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>cta</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>CONTACT_US</t>
         </is>
@@ -2265,6 +2570,511 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:T5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="23" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="16" max="16"/>
+    <col width="19" customWidth="1" min="17" max="17"/>
+    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="38" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>audience_key</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>account_key</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>meta_audience_id</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>audience_type</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>subtype</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>source_audience_key</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>pixel_dataset_id</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>retention_days</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>countries</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>lookalike_ratio</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>targeting_json</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>rule_json</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>lookalike_spec_json</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>customer_file_source</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>approval_status</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>last_result</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>last_error</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>aud_vip_buyers</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>acct_demo_us</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>VIP Buyers Seed</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>CUSTOM</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>CUSTOM</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Seed audience for customers uploaded from CRM.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="3" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>USER_PROVIDED_ONLY</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="R2" s="4" t="inlineStr"/>
+      <c r="S2" s="4" t="inlineStr"/>
+      <c r="T2" s="4" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>aud_vip_lookalike_us</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>acct_demo_us</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>VIP Buyers Lookalike 1% US</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>LOOKALIKE</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>LOOKALIKE</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>US lookalike based on VIP buyers seed.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>aud_vip_buyers</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>{"type":"similarity","ratio":0.01,"country":"US"}</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr"/>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="R3" s="4" t="inlineStr"/>
+      <c r="S3" s="4" t="inlineStr"/>
+      <c r="T3" s="4" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>aud_site_visitors_30d</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>acct_demo_us</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Site Visitors 30D</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>WEBSITE</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>WEBSITE</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Recent website visitors from the demo pixel.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>998877665544</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>{"inclusions":{"operator":"or","rules":[{"event_sources":[{"id":"998877665544","type":"pixel"}],"retention_seconds":2592000,"filter":{"operator":"and","filters":[{"field":"event","operator":"eq","value":"PageView"}]}}]}}</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="R4" s="4" t="inlineStr"/>
+      <c r="S4" s="4" t="inlineStr"/>
+      <c r="T4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>aud_saved_broad_us</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>acct_demo_us</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Saved Broad US 25-54</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>SAVED</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Reusable broad saved audience.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="3" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>{"geo_locations":{"countries":["US"]},"age_min":25,"age_max":54}</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr"/>
+      <c r="O5" s="2" t="inlineStr"/>
+      <c r="P5" s="2" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="R5" s="4" t="inlineStr"/>
+      <c r="S5" s="4" t="inlineStr"/>
+      <c r="T5" s="4" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="38" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>upload_key</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>audience_key</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>operation</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>schema</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>data_path</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>data_json</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>hash_type</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>approval_status</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>applied_at</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>result</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>upload_vip_buyers_seed</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>aud_vip_buyers</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>EMAIL,FN,LN</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>audience_uploads/vip_buyers.csv</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>HASHED</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr"/>
+      <c r="J2" s="4" t="inlineStr"/>
+      <c r="K2" s="4" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2523,7 +3333,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2711,174 +3521,4 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>log_id</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>timestamp</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>mode</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>action_id</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>operation</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>object_type</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>object_key</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>meta_id</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>command</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>payload_hash</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>message</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>stdout</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>stderr</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>validation_id</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>timestamp</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>severity</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>table</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>row_key</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>field</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>message</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add duplicate job workflow
</commit_message>
<xml_diff>
--- a/examples/meta_ads_workflow_template.xlsx
+++ b/examples/meta_ads_workflow_template.xlsx
@@ -16,11 +16,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ads" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audiences" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudienceUploads" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BulkChanges" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PerformanceSnapshots" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PublishLog" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ValidationErrors" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookups" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DuplicateJobs" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BulkChanges" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PerformanceSnapshots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PublishLog" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ValidationErrors" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookups" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -197,7 +198,33 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="BulkChangesTable" displayName="BulkChangesTable" ref="A1:M4" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="DuplicateJobsTable" displayName="DuplicateJobsTable" ref="A1:Q3" headerRowCount="1">
+  <autoFilter ref="A1:Q3"/>
+  <tableColumns count="17">
+    <tableColumn id="1" name="job_key"/>
+    <tableColumn id="2" name="object_level"/>
+    <tableColumn id="3" name="source_key_or_meta_id"/>
+    <tableColumn id="4" name="destination_parent_key_or_meta_id"/>
+    <tableColumn id="5" name="copy_count"/>
+    <tableColumn id="6" name="deep_copy"/>
+    <tableColumn id="7" name="status_option"/>
+    <tableColumn id="8" name="rename_strategy"/>
+    <tableColumn id="9" name="name_prefix"/>
+    <tableColumn id="10" name="name_suffix"/>
+    <tableColumn id="11" name="overrides_json"/>
+    <tableColumn id="12" name="create_rows"/>
+    <tableColumn id="13" name="approval_status"/>
+    <tableColumn id="14" name="applied_at"/>
+    <tableColumn id="15" name="result_meta_ids"/>
+    <tableColumn id="16" name="result"/>
+    <tableColumn id="17" name="error"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="BulkChangesTable" displayName="BulkChangesTable" ref="A1:M4" headerRowCount="1">
   <autoFilter ref="A1:M4"/>
   <tableColumns count="13">
     <tableColumn id="1" name="change_id"/>
@@ -218,8 +245,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="PerformanceSnapshotsTable" displayName="PerformanceSnapshotsTable" ref="A1:AB2" headerRowCount="1">
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="PerformanceSnapshotsTable" displayName="PerformanceSnapshotsTable" ref="A1:AB2" headerRowCount="1">
   <autoFilter ref="A1:AB2"/>
   <tableColumns count="28">
     <tableColumn id="1" name="snapshot_key"/>
@@ -255,8 +282,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="PublishLogTable" displayName="PublishLogTable" ref="A1:N2" headerRowCount="1">
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="PublishLogTable" displayName="PublishLogTable" ref="A1:N2" headerRowCount="1">
   <autoFilter ref="A1:N2"/>
   <tableColumns count="14">
     <tableColumn id="1" name="log_id"/>
@@ -278,8 +305,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="ValidationErrorsTable" displayName="ValidationErrorsTable" ref="A1:G2" headerRowCount="1">
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="ValidationErrorsTable" displayName="ValidationErrorsTable" ref="A1:G2" headerRowCount="1">
   <autoFilter ref="A1:G2"/>
   <tableColumns count="7">
     <tableColumn id="1" name="validation_id"/>
@@ -294,9 +321,9 @@
 </table>
 </file>
 
-<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="LookupsTable" displayName="LookupsTable" ref="A1:B27" headerRowCount="1">
-  <autoFilter ref="A1:B27"/>
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="LookupsTable" displayName="LookupsTable" ref="A1:B33" headerRowCount="1">
+  <autoFilter ref="A1:B33"/>
   <tableColumns count="2">
     <tableColumn id="1" name="type"/>
     <tableColumn id="2" name="value"/>
@@ -1021,6 +1048,259 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:Q3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="19" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="19" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="38" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>job_key</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>object_level</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>source_key_or_meta_id</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>destination_parent_key_or_meta_id</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>copy_count</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>deep_copy</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>status_option</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>rename_strategy</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>name_prefix</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>name_suffix</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>overrides_json</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>create_rows</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>approval_status</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>applied_at</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>result_meta_ids</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>result</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>dup_prospecting_ad</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>ad_prospecting_static_a</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>adset_prospecting_us</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>PAUSED</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>APPEND</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | Copy</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="N2" s="4" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="4" t="inlineStr"/>
+      <c r="Q2" s="4" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>dup_retargeting_adset</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>adset</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>adset_retargeting_us</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>cmp_spring_launch</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>PAUSED</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>APPEND</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | Weekend</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>{"start_time":"2026-06-18T09:00:00-04:00","end_time":"2026-06-21T23:59:00-04:00"}</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="N3" s="4" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr"/>
+      <c r="P3" s="4" t="inlineStr"/>
+      <c r="Q3" s="4" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1279,7 +1559,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1469,7 +1749,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1575,7 +1855,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1639,13 +1919,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1931,46 +2211,118 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>cta</t>
+          <t>duplicate_object_level</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>SHOP_NOW</t>
+          <t>campaign</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>cta</t>
+          <t>duplicate_object_level</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>LEARN_MORE</t>
+          <t>adset</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>cta</t>
+          <t>duplicate_object_level</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>SIGN_UP</t>
+          <t>ad</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
+          <t>duplicate_status_option</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>PAUSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>duplicate_status_option</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>duplicate_status_option</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>INHERITED</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
           <t>cta</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>SHOP_NOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>cta</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>LEARN_MORE</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>cta</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>SIGN_UP</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>cta</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>CONTACT_US</t>
         </is>

</xml_diff>

<commit_message>
Expand bulk edits and optimization rules
</commit_message>
<xml_diff>
--- a/examples/meta_ads_workflow_template.xlsx
+++ b/examples/meta_ads_workflow_template.xlsx
@@ -18,10 +18,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudienceUploads" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DuplicateJobs" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BulkChanges" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PerformanceSnapshots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PublishLog" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ValidationErrors" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookups" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OptimizationRules" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PerformanceSnapshots" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PublishLog" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ValidationErrors" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookups" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -224,29 +225,54 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="BulkChangesTable" displayName="BulkChangesTable" ref="A1:M4" headerRowCount="1">
-  <autoFilter ref="A1:M4"/>
-  <tableColumns count="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="BulkChangesTable" displayName="BulkChangesTable" ref="A1:O5" headerRowCount="1">
+  <autoFilter ref="A1:O5"/>
+  <tableColumns count="15">
     <tableColumn id="1" name="change_id"/>
-    <tableColumn id="2" name="object_level"/>
-    <tableColumn id="3" name="object_key_or_meta_id"/>
-    <tableColumn id="4" name="field"/>
-    <tableColumn id="5" name="old_value"/>
-    <tableColumn id="6" name="new_value"/>
-    <tableColumn id="7" name="effective_at"/>
-    <tableColumn id="8" name="reason"/>
-    <tableColumn id="9" name="requested_by"/>
-    <tableColumn id="10" name="approval_status"/>
-    <tableColumn id="11" name="applied_at"/>
-    <tableColumn id="12" name="result"/>
-    <tableColumn id="13" name="error"/>
+    <tableColumn id="2" name="operation"/>
+    <tableColumn id="3" name="object_level"/>
+    <tableColumn id="4" name="object_key_or_meta_id"/>
+    <tableColumn id="5" name="field"/>
+    <tableColumn id="6" name="old_value"/>
+    <tableColumn id="7" name="new_value"/>
+    <tableColumn id="8" name="value_json"/>
+    <tableColumn id="9" name="effective_at"/>
+    <tableColumn id="10" name="reason"/>
+    <tableColumn id="11" name="requested_by"/>
+    <tableColumn id="12" name="approval_status"/>
+    <tableColumn id="13" name="applied_at"/>
+    <tableColumn id="14" name="result"/>
+    <tableColumn id="15" name="error"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="PerformanceSnapshotsTable" displayName="PerformanceSnapshotsTable" ref="A1:AB2" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="OptimizationRulesTable" displayName="OptimizationRulesTable" ref="A1:N3" headerRowCount="1">
+  <autoFilter ref="A1:N3"/>
+  <tableColumns count="14">
+    <tableColumn id="1" name="rule_key"/>
+    <tableColumn id="2" name="scope_level"/>
+    <tableColumn id="3" name="metric"/>
+    <tableColumn id="4" name="operator"/>
+    <tableColumn id="5" name="threshold"/>
+    <tableColumn id="6" name="action_object_level"/>
+    <tableColumn id="7" name="action_field"/>
+    <tableColumn id="8" name="action_value"/>
+    <tableColumn id="9" name="max_actions"/>
+    <tableColumn id="10" name="approval_status"/>
+    <tableColumn id="11" name="generated_change_prefix"/>
+    <tableColumn id="12" name="last_result"/>
+    <tableColumn id="13" name="last_error"/>
+    <tableColumn id="14" name="updated_at"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="PerformanceSnapshotsTable" displayName="PerformanceSnapshotsTable" ref="A1:AB2" headerRowCount="1">
   <autoFilter ref="A1:AB2"/>
   <tableColumns count="28">
     <tableColumn id="1" name="snapshot_key"/>
@@ -282,8 +308,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="PublishLogTable" displayName="PublishLogTable" ref="A1:N2" headerRowCount="1">
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="PublishLogTable" displayName="PublishLogTable" ref="A1:N2" headerRowCount="1">
   <autoFilter ref="A1:N2"/>
   <tableColumns count="14">
     <tableColumn id="1" name="log_id"/>
@@ -305,8 +331,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="ValidationErrorsTable" displayName="ValidationErrorsTable" ref="A1:G2" headerRowCount="1">
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="ValidationErrorsTable" displayName="ValidationErrorsTable" ref="A1:G2" headerRowCount="1">
   <autoFilter ref="A1:G2"/>
   <tableColumns count="7">
     <tableColumn id="1" name="validation_id"/>
@@ -321,8 +347,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="LookupsTable" displayName="LookupsTable" ref="A1:B33" headerRowCount="1">
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="LookupsTable" displayName="LookupsTable" ref="A1:B33" headerRowCount="1">
   <autoFilter ref="A1:B33"/>
   <tableColumns count="2">
     <tableColumn id="1" name="type"/>
@@ -1301,22 +1327,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="38" customWidth="1" min="13" max="13"/>
+    <col width="38" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="38" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1327,60 +1355,70 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>operation</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>object_level</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>object_key_or_meta_id</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>field</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>old_value</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>new_value</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>value_json</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>effective_at</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>reason</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>requested_by</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>approval_status</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>applied_at</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>result</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>error</t>
         </is>
@@ -1394,52 +1432,58 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>SET_FIELD</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
           <t>campaign</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>cmp_spring_launch</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>daily_budget_cents</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>5000</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>7500</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>2026-06-04T09:00:00-04:00</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Increase launch-day budget after creative QA.</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Growth Team</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>APPROVED</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr"/>
-      <c r="L2" s="4" t="inlineStr"/>
       <c r="M2" s="4" t="inlineStr"/>
+      <c r="N2" s="4" t="inlineStr"/>
+      <c r="O2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1449,52 +1493,58 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>SET_FIELD</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
           <t>adset</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>adset_prospecting_us</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>bid_amount_cents</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>1200</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>1500</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>2026-06-04T09:00:00-04:00</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Raise bid cap to improve launch delivery.</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Growth Team</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>APPROVED</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr"/>
-      <c r="L3" s="4" t="inlineStr"/>
       <c r="M3" s="4" t="inlineStr"/>
+      <c r="N3" s="4" t="inlineStr"/>
+      <c r="O3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1504,52 +1554,111 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
+          <t>SET_FIELD</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
           <t>adset</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>adset_retargeting_us</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>end_time</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>2026-06-17T23:59:00-04:00</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>2026-06-21T23:59:00-04:00</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>2026-06-10T09:00:00-04:00</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>Extend retargeting window through final promo weekend.</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Growth Team</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>APPROVED</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr"/>
-      <c r="L4" s="4" t="inlineStr"/>
       <c r="M4" s="4" t="inlineStr"/>
+      <c r="N4" s="4" t="inlineStr"/>
+      <c r="O4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>chg_patch_retargeting_targeting</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>PATCH_JSON</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>adset</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>adset_retargeting_us</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>{"targeting_automation":{"advantage_audience":0}}</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04T09:00:00-04:00</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Force manual retargeting controls for the demo ad set.</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Growth Team</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr"/>
+      <c r="N5" s="4" t="inlineStr"/>
+      <c r="O5" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1560,6 +1669,231 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="27" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="38" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rule_key</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>scope_level</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>operator</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>threshold</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>action_object_level</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>action_field</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>action_value</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>max_actions</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>approval_status</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>generated_change_prefix</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>last_result</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>last_error</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>pause_high_cpa_ads</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>cost_per_result</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>desired_status</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>PAUSED</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>opt_pause_high_cpa</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr"/>
+      <c r="M2" s="4" t="inlineStr"/>
+      <c r="N2" s="4" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>raise_budget_high_roas_campaigns</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>roas</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>&gt;=</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>campaign</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>daily_budget_cents</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>9000</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>opt_raise_budget</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr"/>
+      <c r="M3" s="4" t="inlineStr"/>
+      <c r="N3" s="4" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1749,7 +2083,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1855,7 +2189,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1919,7 +2253,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Expand insights and document workflow coverage
</commit_message>
<xml_diff>
--- a/examples/meta_ads_workflow_template.xlsx
+++ b/examples/meta_ads_workflow_template.xlsx
@@ -272,9 +272,9 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="PerformanceSnapshotsTable" displayName="PerformanceSnapshotsTable" ref="A1:AB2" headerRowCount="1">
-  <autoFilter ref="A1:AB2"/>
-  <tableColumns count="28">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="PerformanceSnapshotsTable" displayName="PerformanceSnapshotsTable" ref="A1:AK2" headerRowCount="1">
+  <autoFilter ref="A1:AK2"/>
+  <tableColumns count="37">
     <tableColumn id="1" name="snapshot_key"/>
     <tableColumn id="2" name="date"/>
     <tableColumn id="3" name="object_level"/>
@@ -282,27 +282,36 @@
     <tableColumn id="5" name="campaign_key"/>
     <tableColumn id="6" name="adset_key"/>
     <tableColumn id="7" name="ad_key"/>
-    <tableColumn id="8" name="spend"/>
-    <tableColumn id="9" name="impressions"/>
-    <tableColumn id="10" name="reach"/>
-    <tableColumn id="11" name="frequency"/>
-    <tableColumn id="12" name="clicks"/>
-    <tableColumn id="13" name="link_clicks"/>
-    <tableColumn id="14" name="landing_page_views"/>
-    <tableColumn id="15" name="ctr"/>
-    <tableColumn id="16" name="cpc"/>
-    <tableColumn id="17" name="cpm"/>
-    <tableColumn id="18" name="conversions"/>
-    <tableColumn id="19" name="cost_per_result"/>
-    <tableColumn id="20" name="purchases"/>
-    <tableColumn id="21" name="purchase_value"/>
-    <tableColumn id="22" name="roas"/>
-    <tableColumn id="23" name="add_to_cart"/>
-    <tableColumn id="24" name="initiate_checkout"/>
-    <tableColumn id="25" name="leads"/>
-    <tableColumn id="26" name="cpl"/>
-    <tableColumn id="27" name="budget_utilization"/>
-    <tableColumn id="28" name="pacing_ratio"/>
+    <tableColumn id="8" name="breakdown_type"/>
+    <tableColumn id="9" name="breakdown_value"/>
+    <tableColumn id="10" name="publisher_platform"/>
+    <tableColumn id="11" name="platform_position"/>
+    <tableColumn id="12" name="country"/>
+    <tableColumn id="13" name="region"/>
+    <tableColumn id="14" name="age"/>
+    <tableColumn id="15" name="gender"/>
+    <tableColumn id="16" name="device_platform"/>
+    <tableColumn id="17" name="spend"/>
+    <tableColumn id="18" name="impressions"/>
+    <tableColumn id="19" name="reach"/>
+    <tableColumn id="20" name="frequency"/>
+    <tableColumn id="21" name="clicks"/>
+    <tableColumn id="22" name="link_clicks"/>
+    <tableColumn id="23" name="landing_page_views"/>
+    <tableColumn id="24" name="ctr"/>
+    <tableColumn id="25" name="cpc"/>
+    <tableColumn id="26" name="cpm"/>
+    <tableColumn id="27" name="conversions"/>
+    <tableColumn id="28" name="cost_per_result"/>
+    <tableColumn id="29" name="purchases"/>
+    <tableColumn id="30" name="purchase_value"/>
+    <tableColumn id="31" name="roas"/>
+    <tableColumn id="32" name="add_to_cart"/>
+    <tableColumn id="33" name="initiate_checkout"/>
+    <tableColumn id="34" name="leads"/>
+    <tableColumn id="35" name="cpl"/>
+    <tableColumn id="36" name="budget_utilization"/>
+    <tableColumn id="37" name="pacing_ratio"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1899,7 +1908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AK2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1909,27 +1918,36 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="15" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="19" customWidth="1" min="16" max="16"/>
     <col width="14" customWidth="1" min="17" max="17"/>
     <col width="15" customWidth="1" min="18" max="18"/>
-    <col width="19" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="18" customWidth="1" min="21" max="21"/>
-    <col width="14" customWidth="1" min="22" max="22"/>
-    <col width="15" customWidth="1" min="23" max="23"/>
-    <col width="21" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="15" customWidth="1" min="22" max="22"/>
+    <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
     <col width="14" customWidth="1" min="25" max="25"/>
     <col width="14" customWidth="1" min="26" max="26"/>
-    <col width="22" customWidth="1" min="27" max="27"/>
-    <col width="16" customWidth="1" min="28" max="28"/>
+    <col width="15" customWidth="1" min="27" max="27"/>
+    <col width="19" customWidth="1" min="28" max="28"/>
+    <col width="14" customWidth="1" min="29" max="29"/>
+    <col width="18" customWidth="1" min="30" max="30"/>
+    <col width="14" customWidth="1" min="31" max="31"/>
+    <col width="15" customWidth="1" min="32" max="32"/>
+    <col width="21" customWidth="1" min="33" max="33"/>
+    <col width="14" customWidth="1" min="34" max="34"/>
+    <col width="14" customWidth="1" min="35" max="35"/>
+    <col width="22" customWidth="1" min="36" max="36"/>
+    <col width="16" customWidth="1" min="37" max="37"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1970,105 +1988,150 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>breakdown_type</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>breakdown_value</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>publisher_platform</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>platform_position</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>region</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>age</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>gender</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>device_platform</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>spend</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>impressions</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>reach</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>frequency</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>clicks</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>link_clicks</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>landing_page_views</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>ctr</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>cpc</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>cpm</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>conversions</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>cost_per_result</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>purchases</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>purchase_value</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>roas</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>add_to_cart</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>initiate_checkout</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>leads</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>cpl</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>budget_utilization</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>pacing_ratio</t>
         </is>

</xml_diff>